<commit_message>
final version all ai camera stability map and web done
</commit_message>
<xml_diff>
--- a/fiche robot price and ref.xlsx
+++ b/fiche robot price and ref.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ysxay\Documents\1st robot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ysxay\Documents\1st-robot\3D-model\my-first-hardware-robot-yaya\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5B41A2-BED4-468C-B43D-C6A667D6D72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3ED0D9-0D8A-4032-ADE9-12D6D5264525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{5385AF8B-5E78-4C05-9C0A-C88B91E9E402}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="116">
   <si>
     <t>servo motor</t>
   </si>
@@ -146,9 +146,6 @@
     <t>https://www.amazon.fr/GERUI-cartes-d%C3%A9rivation-multiplexeur-TCA9548A/dp/B0F37Y8HWV/ref=sr_1_1?__mk_fr_FR=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=31BKDCG1A75O8&amp;dib=eyJ2IjoiMSJ9.39RdYhq796rUa1hmQbSVM5nTyrkZYy0xg3WK52CaZMYKKdGMf95TproMTYPgRYlD62_YDFHD4pajETiRhFOBRqvvmMvs3hBU0dQsNWdUtHj3HSbUaVX8UR2Q_0hfLS0UTnxup76vrbvlJUqRHkRyecE-4BdLvVMebieToqz0tpLwAt_mCLmm7eJw_KHXzzlZbiJx0g4aKqn5q8QQbJHKwxf2sWTogSms8Yh8fBI2ov2gpouPfMiLtpeg_c39zoJaX7Fmiw3188P2W5PEpRH5PpUrpqBPgIBmw1YnFkTdYQ8.VZqaTNt1bNF_JpYtU_-xO4ZZP-FrwE85MI7_704bRU8&amp;dib_tag=se&amp;keywords=Module+multiplexeur+I2C+DFR0576+%C3%A0+8+canaux+Module+multiplexeur+I2C+bas%C3%A9+sur+un+TCA9548A+permettant+de+raccorder+jusqu%27%C3%A0+8+capteurs+I2C+avec+la+m%C3%AAme+adresse+sur+le+m%C3%AAme+bus+I2C+d%27un+microcontr%C3%B4leur.+8%2C90+%E2%82%AC+TTC+7%2C42+%E2%82%AC+HT+Code+%3A+36123&amp;qid=1784153675&amp;sprefix=module+multiplexeur+i2c+dfr0576+%C3%A0+8+canaux+module+multiplexeur+i2c+bas%C3%A9+sur+un+tca9548a+permettant+de+raccorder+jusqu%27%C3%A0+8+capteurs+i2c+avec+la+m%C3%AAme+adresse+sur+le+m%C3%AAme+bus+i2c+d%27un+microcontr%C3%B4leur.+8%2C90+ttc+7%2C42+ht+code+36123%2Caps%2C199&amp;sr=8-1</t>
   </si>
   <si>
-    <t>https://www.gotronic.fr/art-capteur-de-distance-tof-48876.htm</t>
-  </si>
-  <si>
     <t>Module 9 DoF BNO055</t>
   </si>
   <si>
@@ -179,9 +176,6 @@
     <t>https://www.amazon.fr/servomoteurs-encodeur-magn%C3%A9tique-pr%C3%A9cision-%C3%A9ducatifs/dp/B0FLPQQ4FR/ref=sr_1_1?__mk_fr_FR=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=EK8QST769I4K&amp;dib=eyJ2IjoiMSJ9.bO0-KRlSPeQgqdTs_BShPCEHgHZIJ3MqCN2454hsiQau6HUxctjsLQOICXFTwoRdmtygxTpaFs37Hou155x1HZFhxNKL3MGNYfJO3pJH7QxEaKA8vDMXKwkdtzMM9feqb00oMigKdlfHW00afriBAHXYlXgOHaGRzLpJCsVrd9luwtEllAdqAjSwCOq7yfQz.TVMFxZFUHGvQf2jKWUSC_IDa0M7urx4bHnKuH2JCxjo&amp;dib_tag=se&amp;keywords=rcmall+feetech+sts3215+12v+30kg+lot+6+servomoteur&amp;qid=1784163563&amp;sprefix=rcmall+feetech+sts3215+12v+30kg+lot+6+servomoteurs%2Caps%2C187&amp;sr=8-1&amp;ufe=app_do%3Aamzn1.fos.49fccda8-a887-4188-817b-b9a64bb30e43</t>
   </si>
   <si>
-    <t>Capteur de distance VL53L1X 333064 x3</t>
-  </si>
-  <si>
     <t>oled (pure looks)</t>
   </si>
   <si>
@@ -225,12 +219,6 @@
   </si>
   <si>
     <t>camera raspberry adaotator</t>
-  </si>
-  <si>
-    <t>https://www.kubii.com/fr/nappes-cables-adaptateurs/4116-1860-nappe-csi-mipi-camera-pour-raspberry-pi-5-3272496316669.html</t>
-  </si>
-  <si>
-    <t>Nappe CSI / MIPI caméra pour Raspberry Pi 5</t>
   </si>
   <si>
     <t xml:space="preserve">  </t>
@@ -333,12 +321,6 @@
     <t>https://www.amazon.fr/Elegoo-Breadboard-Femelle-Longueur-Arduino/dp/B01JD5WCG2/ref=sr_1_2_sspa?__mk_fr_FR=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=3JOJRK0HMI602&amp;dib=eyJ2IjoiMSJ9.cjmjAB8qRNR9Llwct3Zm97Aqo2A0HAgzQaA1b2Aq9uYW8ULfWXfXo10D8AAMde0vyD_YgVaP2W5jQexhdbupMWziEBnJLBrotK4IxoJ-NdKIM5KgutYZcZ1s1iJuUmOukK4yOUoi_t3uqPJRRad0xVbAjkuEnpJL0XMaOd9VYy6s2hCLopmKEVJ8HBaP16bI_YC3PeIlqWSfwO7zG5Al_s7ycMFDEzSxiKgbavldiO62R2u4p75fieQhm9BsHatjAlxOXhKWC0BezHz2Aw1O0OD0yYWNE4R6k0wNUq54R9M.ZrF5cVuyhKWn0xv0Z7QQybRsD5pSABfWzEUEHtHMvFI&amp;dib_tag=se&amp;keywords=fil+dupont&amp;qid=1785355088&amp;s=industrial&amp;sprefix=fil+dupon%2Cindustrial%2C227&amp;sr=1-2-spons&amp;aref=pTIwZ5WZPw&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
   </si>
   <si>
-    <t>2.4 pouce SD1309 128x64</t>
-  </si>
-  <si>
-    <t>https://www.amazon.com/dp/B0GTPS8JR7?th=1</t>
-  </si>
-  <si>
     <t>adaptator radxa</t>
   </si>
   <si>
@@ -367,6 +349,42 @@
   </si>
   <si>
     <t>usb-c to usb-c x 2 data en charge</t>
+  </si>
+  <si>
+    <t>speaker kit</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0GV33LRR5?lv=shuf&amp;channelId=500&amp;plpRedirect=mhFallback&amp;th=1</t>
+  </si>
+  <si>
+    <t>kit I2S audio amplifer + speaker</t>
+  </si>
+  <si>
+    <t>ldar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stt </t>
+  </si>
+  <si>
+    <t>microphone</t>
+  </si>
+  <si>
+    <t>https://www.amazon.fr/Microphone-Omnidirectionnel-Enregistrement-Transmission-Electrique/dp/B0GYYQBS34/ref=sr_1_1_sspa?adgrpid=62171879496&amp;dib=eyJ2IjoiMSJ9.brjZqMMDrrRHvnt_m92c34XSqXmV6OV8aO_jOHQzQEJoo9L83dbjyDPmZu-9vNcwBCad-wm0-8rAalVFW68LukKTDbUAHGbDvZdPtU0Knoflk8QT5s1Wd4_b3UiflWXi2LAk6CqeB4mHHXD6hPf3BWNeDmNnerYjqSSUHs_mF8k-ED93Ze0C-jmlsoUYKJf38KapQQ4NLf_QJS3cHoogIp2CgQh2GXM0Rn3bNnv1HbZxrxbD8NlIImi2g2g6TfXHPQzhZmiejd5I8zpEfz_nnJYNQKpgDGFFcj3pRuLrZP0.rojuTPoUDQE2-asi-jPvjvAcJTd5-AH8Wpvfk8cW4jw&amp;dib_tag=se&amp;hvadid=310714367915&amp;hvdev=c&amp;hvexpln=0&amp;hvlocphy=9055055&amp;hvnetw=g&amp;hvocijid=1494477379405652865--&amp;hvqmt=e&amp;hvrand=1494477379405652865&amp;hvtargid=kwd-528219262780&amp;hydadcr=14030_1730247&amp;keywords=inmp441&amp;mcid=0a7caf62588f36e7bcadcf677d060076&amp;qid=1786228193&amp;sr=8-1-spons&amp;aref=YFzPhMXmpy&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1</t>
+  </si>
+  <si>
+    <t>https://www.gotronic.fr/art-capteur-de-distance-rplidar-a1m8-29031.htm</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0DQBHNT9C?lv=shuf&amp;channelId=500&amp;plpRedirect=mhFallback</t>
+  </si>
+  <si>
+    <t>Nappe CSI / MIPI 15 to 22 30cm</t>
+  </si>
+  <si>
+    <t>https://www.amazon.fr/Helilyco-%C3%89cran-Arduino-%C3%A9cran-esp32/dp/B0H71WGG1S/ref=sr_1_5?dib=eyJ2IjoiMSJ9.jdwm-TZBxVLh94ZZ6vdGqkd0IDZyWgyI5k35lOhz0Rqs2-ERSIOIV6dX7_JQHov_mUNFY8cUMQzvEmGn9a99Pn8P9s9tHme_BT2SJNMd7Lj_vWF61ICik9WixTCkjNFynJ9A4CLs8ZY_V6hdYcMBypCWwRTDSoGC0D08dJDKqSP16ezMpnZjBmKSaDxYJIvvhG13kHSV0hf0y4s5TzENkchtSzIRhupK-RzV1Ewv7VmkHYEuFFg7Ej3L-0MpVSPJOf13TrUUwRDuvKuRQyTK5NX72SAApJO4Y5-bvVu5w9w.atJvDhClP-y_iAZagxuVesYT1XkKdKvbQ4Xun9vkWqQ&amp;dib_tag=se&amp;keywords=oled%2B128x64&amp;qid=1786820824&amp;refinements=p_36%3A-1000&amp;rnid=2492331031&amp;sr=8-5&amp;th=1</t>
+  </si>
+  <si>
+    <t>0.96 pouc 128x64</t>
   </si>
 </sst>
 </file>
@@ -808,7 +826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{008D84E1-5605-4D40-8D4F-5DD6771B34B3}">
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
@@ -841,28 +859,28 @@
         <v>0</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C4">
         <f>PRODUCT(146*2)</f>
         <v>292</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C5">
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -942,55 +960,55 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C16">
         <v>56</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
         <v>44</v>
-      </c>
-      <c r="B17" t="s">
-        <v>45</v>
       </c>
       <c r="C17">
         <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B18" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C18">
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C19">
         <v>10</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1012,13 +1030,13 @@
         <v>10</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C29">
         <v>32</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
@@ -1026,13 +1044,13 @@
         <v>11</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="C30">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>36</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
@@ -1051,357 +1069,386 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B32" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C32">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B33" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C33">
         <v>35</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>64</v>
+        <v>113</v>
       </c>
       <c r="C34">
-        <v>2.4</v>
+        <v>9</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>63</v>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B35" t="s">
+        <v>106</v>
+      </c>
+      <c r="C35">
+        <v>9</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
+        <v>108</v>
+      </c>
+      <c r="B36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36">
+        <v>9</v>
+      </c>
+      <c r="D36" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>3</v>
       </c>
-      <c r="C36">
-        <f>SUM(C29:C34)</f>
-        <v>133.4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>19</v>
+      <c r="C38">
+        <f>SUM(C29:C36)</f>
+        <v>227</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>107</v>
-      </c>
-      <c r="B41" t="s">
-        <v>109</v>
-      </c>
-      <c r="C41">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43">
         <f>PRODUCT(8,2)</f>
         <v>16</v>
       </c>
-      <c r="D41" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="D43" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>21</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B44" t="s">
         <v>22</v>
-      </c>
-      <c r="C42">
-        <v>17</v>
-      </c>
-      <c r="D42" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>100</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C43">
-        <v>17</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="28" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>30</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="C44">
         <v>17</v>
       </c>
       <c r="D44" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>39</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>79</v>
+        <v>94</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>80</v>
       </c>
       <c r="C45">
         <v>17</v>
       </c>
-      <c r="D45" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D45" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>30</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C46">
+        <v>17</v>
+      </c>
+      <c r="D46" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="28" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>76</v>
+        <v>38</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>75</v>
       </c>
       <c r="C47">
-        <v>7</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>86</v>
-      </c>
-      <c r="B48" t="s">
-        <v>88</v>
-      </c>
-      <c r="C48">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s">
-        <v>87</v>
+        <v>17</v>
+      </c>
+      <c r="D47" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>91</v>
-      </c>
-      <c r="B49" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="C49">
-        <v>18</v>
-      </c>
-      <c r="D49" t="s">
-        <v>93</v>
+        <v>7</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="B50" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C50">
         <v>9</v>
       </c>
       <c r="D50" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51">
+        <v>18</v>
+      </c>
+      <c r="D51" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" t="s">
+        <v>92</v>
+      </c>
+      <c r="C52">
+        <v>9</v>
+      </c>
+      <c r="D52" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>3</v>
       </c>
-      <c r="C51">
-        <f>SUM(C40:C50)</f>
+      <c r="C53">
+        <f>SUM(C42:C52)</f>
         <v>127</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>51</v>
-      </c>
-      <c r="B56" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>57</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C57">
-        <v>10</v>
-      </c>
-      <c r="D57" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B58" t="s">
-        <v>75</v>
-      </c>
-      <c r="C58">
-        <v>2.4</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
+        <v>55</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C59">
+        <v>10</v>
+      </c>
+      <c r="D59" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>50</v>
+      </c>
+      <c r="B60" t="s">
+        <v>71</v>
+      </c>
+      <c r="C60">
+        <v>2.4</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>62</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C61">
+        <v>20</v>
+      </c>
+      <c r="D61" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>66</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B62" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C62">
+        <v>10</v>
+      </c>
+      <c r="D62" t="s">
         <v>67</v>
       </c>
-      <c r="C59">
-        <v>20</v>
-      </c>
-      <c r="D59" t="s">
+    </row>
+    <row r="63" spans="1:4" ht="28" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+      <c r="B63" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="C63">
+        <v>14</v>
+      </c>
+      <c r="D63" t="s">
         <v>69</v>
       </c>
-      <c r="C60">
-        <v>10</v>
-      </c>
-      <c r="D60" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="28" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>72</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C61">
-        <v>14</v>
-      </c>
-      <c r="D61" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>53</v>
-      </c>
-      <c r="B62" t="s">
-        <v>55</v>
-      </c>
-      <c r="C62">
-        <v>0</v>
-      </c>
-      <c r="D62" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D63" s="1"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
+        <v>51</v>
+      </c>
+      <c r="B64" t="s">
+        <v>53</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
+      <c r="D64" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D65" s="1"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>3</v>
       </c>
-      <c r="C64">
-        <f>SUM(C57:C63)</f>
+      <c r="C66">
+        <f>SUM(C59:C65)</f>
         <v>56.4</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="C71" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C73" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>39</v>
+      </c>
+      <c r="B74" t="s">
         <v>40</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C74">
+        <f>SUM(C6,C13,C25,C38,C53,C66,)</f>
+        <v>847.4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>42</v>
+      </c>
+      <c r="B75" t="s">
         <v>41</v>
-      </c>
-      <c r="C72">
-        <f>SUM(C6,C13,C25,C36,C51,C64,)</f>
-        <v>753.8</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>43</v>
-      </c>
-      <c r="B73" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D32" r:id="rId1" xr:uid="{9289B590-F30A-4593-9C30-D7D41A61602F}"/>
+    <hyperlink ref="D32" r:id="rId1" display="https://www.amazon.com/dp/B0GTPS8JR7?th=1" xr:uid="{9289B590-F30A-4593-9C30-D7D41A61602F}"/>
     <hyperlink ref="D9" r:id="rId2" xr:uid="{B8E574BC-7EDC-4E8F-A62E-3439BFFEFF11}"/>
     <hyperlink ref="D29" r:id="rId3" xr:uid="{A0752B03-C1AE-41B4-A816-A07488D6544D}"/>
-    <hyperlink ref="D43" r:id="rId4" display="https://www.amazon.fr/Convertisseur-Binghe-Reconnaissance-Compatible-Arduino/dp/B0DJX9GVX6/ref=sr_1_5_sspa?__mk_fr_FR=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=HQQ8XQUDPPHV&amp;dib=eyJ2IjoiMSJ9.kFvMDwPnhb169LU9cfq_j6Az3BvHQE5mAWWiirbf3OeW2J6pNaifAlx6Hyu-CaFiyeJcUP3ZfkN8VmXvsfUKKVCBlt5DKaFItbLPtFh_vYK84-EH2y4Z-mex-sqrcv4L7Xdm4GjlZn9b10Z5x-TYyznWMo8kJhCMFQs08EZeWL2eYHNlfYMd3abtAz166thI799K3VE3BfWi-FnHvJ4g9fGqxuoif2ddb77mcIKNZr8x3uTCUKFCFBlMZfZI8HgWm9mIYf5-vE74WhLoHE66SCRAs2V2aupT8_JC1gAxy2w.zHIm-JR1-VSmU9ObNOCcP07cP8JLhJOviBAAb1VbyuU&amp;dib_tag=se&amp;keywords=buck+converter+12v+to+5v&amp;qid=1785351091&amp;sprefix=buck+converter+12v+to+5v%2Caps%2C192&amp;sr=8-5-spons&amp;aref=JMKHTNNt9C&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{CC730371-9F52-4255-965E-01643FFC55A2}"/>
+    <hyperlink ref="D45" r:id="rId4" display="https://www.amazon.fr/Convertisseur-Binghe-Reconnaissance-Compatible-Arduino/dp/B0DJX9GVX6/ref=sr_1_5_sspa?__mk_fr_FR=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=HQQ8XQUDPPHV&amp;dib=eyJ2IjoiMSJ9.kFvMDwPnhb169LU9cfq_j6Az3BvHQE5mAWWiirbf3OeW2J6pNaifAlx6Hyu-CaFiyeJcUP3ZfkN8VmXvsfUKKVCBlt5DKaFItbLPtFh_vYK84-EH2y4Z-mex-sqrcv4L7Xdm4GjlZn9b10Z5x-TYyznWMo8kJhCMFQs08EZeWL2eYHNlfYMd3abtAz166thI799K3VE3BfWi-FnHvJ4g9fGqxuoif2ddb77mcIKNZr8x3uTCUKFCFBlMZfZI8HgWm9mIYf5-vE74WhLoHE66SCRAs2V2aupT8_JC1gAxy2w.zHIm-JR1-VSmU9ObNOCcP07cP8JLhJOviBAAb1VbyuU&amp;dib_tag=se&amp;keywords=buck+converter+12v+to+5v&amp;qid=1785351091&amp;sprefix=buck+converter+12v+to+5v%2Caps%2C192&amp;sr=8-5-spons&amp;aref=JMKHTNNt9C&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{CC730371-9F52-4255-965E-01643FFC55A2}"/>
     <hyperlink ref="D34" r:id="rId5" xr:uid="{FE7A531F-AAA0-4944-A62B-0602CF337946}"/>
-    <hyperlink ref="D58" r:id="rId6" xr:uid="{2C573CFC-B095-4D27-8EFA-A474BEAC73AE}"/>
+    <hyperlink ref="D60" r:id="rId6" xr:uid="{2C573CFC-B095-4D27-8EFA-A474BEAC73AE}"/>
     <hyperlink ref="D30" r:id="rId7" xr:uid="{EE78AE99-F2A4-47C9-8866-6600AEDD9D7A}"/>
     <hyperlink ref="D16" r:id="rId8" xr:uid="{402AD104-0565-40F3-B0E3-E1836717E949}"/>
-    <hyperlink ref="D47" r:id="rId9" display="https://www.amazon.fr/Connecteur-Batterie-Voitures-Panneaux-Solaires/dp/B0FS1GLND9/ref=sr_1_1_sspa?dib=eyJ2IjoiMSJ9.zziqtRqTCZHFpD9zjSpZVFtxCCfnnRgFxksWnknbxn1GRH1UJ6XpJtt_Vcu8ADqOnQna2B2yiNtsRKtvAK6LwIWeN9X_hEDqseBW0A_fiPR9l6DS8Wc2rom16NN6PnCzfM4ScBc4anrZYYGjknPjUDgcD7HUZinc62Axj1rsbLkoZd23G-WrX0rE3tgbCObraIrzWAPel4HExlAUcmYLfUayg5dWkhsrpbPLXCYvqHBJHL4VUs9RHrPKzGoDsqwi-9hAi6nBiMljIIqQch-w0pW69gGtM288_YyI0XJ02b8.8HMfizOuaLkOGqrsoJ6HH3iXYA0Rvxn1Ls6WQmr4myE&amp;dib_tag=se&amp;keywords=Male+Xt60+Connector&amp;qid=1784586789&amp;sr=8-1-spons&amp;aref=xOMZOQT4kc&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{84CD557D-1F3C-4522-BE06-90E88C611D42}"/>
+    <hyperlink ref="D49" r:id="rId9" display="https://www.amazon.fr/Connecteur-Batterie-Voitures-Panneaux-Solaires/dp/B0FS1GLND9/ref=sr_1_1_sspa?dib=eyJ2IjoiMSJ9.zziqtRqTCZHFpD9zjSpZVFtxCCfnnRgFxksWnknbxn1GRH1UJ6XpJtt_Vcu8ADqOnQna2B2yiNtsRKtvAK6LwIWeN9X_hEDqseBW0A_fiPR9l6DS8Wc2rom16NN6PnCzfM4ScBc4anrZYYGjknPjUDgcD7HUZinc62Axj1rsbLkoZd23G-WrX0rE3tgbCObraIrzWAPel4HExlAUcmYLfUayg5dWkhsrpbPLXCYvqHBJHL4VUs9RHrPKzGoDsqwi-9hAi6nBiMljIIqQch-w0pW69gGtM288_YyI0XJ02b8.8HMfizOuaLkOGqrsoJ6HH3iXYA0Rvxn1Ls6WQmr4myE&amp;dib_tag=se&amp;keywords=Male+Xt60+Connector&amp;qid=1784586789&amp;sr=8-1-spons&amp;aref=xOMZOQT4kc&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;psc=1" xr:uid="{84CD557D-1F3C-4522-BE06-90E88C611D42}"/>
     <hyperlink ref="D19" r:id="rId10" xr:uid="{46B228BB-7079-4FD4-BF47-B3BFC5C94962}"/>
-    <hyperlink ref="D41" r:id="rId11" xr:uid="{7C022256-2C79-4B2F-865F-DB9524102F7C}"/>
+    <hyperlink ref="D43" r:id="rId11" xr:uid="{7C022256-2C79-4B2F-865F-DB9524102F7C}"/>
+    <hyperlink ref="D35" r:id="rId12" xr:uid="{6D570FED-445F-46C4-9FE2-2CFB9C98A555}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId12"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>